<commit_message>
test(contratos): actualizar respuestas y acciones desde PostgreSQL
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T75731054-000003</x:t>
+    <x:t>T096B5447-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T75731054-000005</x:t>
+    <x:t>T096B5447-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(formularios): renovar los contratos HTTP de idiomas
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T096B5447-000003</x:t>
+    <x:t>T045134E4-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T096B5447-000005</x:t>
+    <x:t>T045134E4-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(contratos): renovar las cohortes del cierre de formularios
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T045134E4-000003</x:t>
+    <x:t>T6E90C249-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T045134E4-000005</x:t>
+    <x:t>T6E90C249-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(formularios): actualizar la exportación HTTP de cierre
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T6E90C249-000003</x:t>
+    <x:t>T1D0893C6-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T6E90C249-000005</x:t>
+    <x:t>T1D0893C6-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(forms): actualizar export conjunto verificado
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T1D0893C6-000003</x:t>
+    <x:t>T7C19E4E8-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T1D0893C6-000005</x:t>
+    <x:t>T7C19E4E8-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(contratos): calificar menú y navegación con el export HTTP completo
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T7C19E4E8-000003</x:t>
+    <x:t>T3DC6A6CA-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T7C19E4E8-000005</x:t>
+    <x:t>T3DC6A6CA-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(contratos): actualizar las capturas conjuntas del review
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T3DC6A6CA-000003</x:t>
+    <x:t>TD13AB0E1-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T3DC6A6CA-000005</x:t>
+    <x:t>TD13AB0E1-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(contratos): regenerar la exportación HTTP completa de E1
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>TD13AB0E1-000003</x:t>
+    <x:t>TF9CA655A-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>TD13AB0E1-000005</x:t>
+    <x:t>TF9CA655A-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>

<commit_message>
test(contracts): renovar juntas las cohortes HTTP de catálogos E2
</commit_message>
<xml_diff>
--- a/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
+++ b/src/test/fixtures/forms-responses-http/export-state-approved-d2.xlsx
@@ -42,7 +42,7 @@
     <x:t>date</x:t>
   </x:si>
   <x:si>
-    <x:t>T720C2400-000003</x:t>
+    <x:t>T351587C5-000003</x:t>
   </x:si>
   <x:si>
     <x:t>Sin información</x:t>
@@ -51,7 +51,7 @@
     <x:t>private 2</x:t>
   </x:si>
   <x:si>
-    <x:t>T720C2400-000005</x:t>
+    <x:t>T351587C5-000005</x:t>
   </x:si>
   <x:si>
     <x:t>private 4</x:t>

</xml_diff>